<commit_message>
clearer text cleaning column in the icda-8 workbook
</commit_message>
<xml_diff>
--- a/results/sep9_meeting/2_icda8_code_in_label.xlsx
+++ b/results/sep9_meeting/2_icda8_code_in_label.xlsx
@@ -22,7 +22,7 @@
     <t xml:space="preserve">Model</t>
   </si>
   <si>
-    <t xml:space="preserve">Text</t>
+    <t xml:space="preserve">Text cleaning</t>
   </si>
   <si>
     <t xml:space="preserve">Label content</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">ClinicalBERT</t>
   </si>
   <si>
-    <t xml:space="preserve">base</t>
+    <t xml:space="preserve">none</t>
   </si>
   <si>
     <t xml:space="preserve">code number then the label</t>

</xml_diff>